<commit_message>
update project_tracker.xlsx with weekly timeline
</commit_message>
<xml_diff>
--- a/project_tracker.xlsx
+++ b/project_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huqingyuan314/Graduate/NEU/Course/DS5110/Project/Iteration#02/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B9829E7-0A54-FB42-95D5-3F255C5C7949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E30DDE5-9410-AC4A-908F-5E8C3274733F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="760" windowWidth="30240" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Schedule" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="33">
   <si>
     <t>PROJECT NAME</t>
   </si>
@@ -84,16 +84,7 @@
     <t>Define metrics and find datasets</t>
   </si>
   <si>
-    <t>Complete data cleaning and preprocessing</t>
-  </si>
-  <si>
-    <t>Develop visualizations and dashboard wireframes</t>
-  </si>
-  <si>
     <t>Final dashboard prototype with interactivity</t>
-  </si>
-  <si>
-    <t>Final submission with documentation and presentation</t>
   </si>
   <si>
     <t>Qingyuan Hu</t>
@@ -112,6 +103,27 @@
   </si>
   <si>
     <t>PROJECT MEMBER</t>
+  </si>
+  <si>
+    <t>Debug and evaluation</t>
+  </si>
+  <si>
+    <t>Prepare for presentation</t>
+  </si>
+  <si>
+    <t>Final submission with report and documentation</t>
+  </si>
+  <si>
+    <t>Develop dashboard wireframes</t>
+  </si>
+  <si>
+    <t>Develop visualizations</t>
+  </si>
+  <si>
+    <t>Provide interfaces for front/back ends</t>
+  </si>
+  <si>
+    <t>Data cleaning and preprocessing</t>
   </si>
 </sst>
 </file>
@@ -152,7 +164,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -204,6 +216,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -220,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -273,17 +291,26 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -587,11 +614,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.83203125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" style="3" customWidth="1"/>
     <col min="3" max="3" width="17.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" style="3" customWidth="1"/>
     <col min="5" max="5" width="18" style="3" customWidth="1"/>
@@ -601,25 +628,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="19" x14ac:dyDescent="0.2">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
@@ -631,10 +658,10 @@
         <v>18</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
@@ -646,10 +673,10 @@
         <v>1</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
@@ -721,7 +748,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="18" t="s">
         <v>15</v>
       </c>
       <c r="B9" s="11" t="s">
@@ -742,19 +769,19 @@
       <c r="G9" s="7"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="24">
         <v>45810</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="24">
         <v>45817</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="23">
         <v>7</v>
       </c>
       <c r="F10" s="13" t="s">
@@ -763,11 +790,11 @@
       <c r="G10" s="7"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="20" t="s">
+      <c r="A11" s="18" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="C11" s="12">
         <v>45817</v>
@@ -778,68 +805,68 @@
       <c r="E11" s="11">
         <v>7</v>
       </c>
-      <c r="F11" s="14" t="s">
+      <c r="F11" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="7"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="24">
+        <v>45824</v>
+      </c>
+      <c r="D12" s="24">
+        <v>45831</v>
+      </c>
+      <c r="E12" s="23">
+        <v>7</v>
+      </c>
+      <c r="F12" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="G11" s="7"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="12">
-        <v>45824</v>
-      </c>
-      <c r="D12" s="12">
+      <c r="G12" s="7"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="12">
+        <v>45831</v>
+      </c>
+      <c r="D13" s="12">
         <v>45838</v>
       </c>
-      <c r="E12" s="11">
-        <v>14</v>
-      </c>
-      <c r="F12" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="7"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="12">
+      <c r="E13" s="11">
+        <v>7</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="7"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="24">
         <v>45838</v>
       </c>
-      <c r="D13" s="12">
-        <v>45852</v>
-      </c>
-      <c r="E13" s="11">
-        <v>14</v>
-      </c>
-      <c r="F13" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="7"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="20" t="s">
-        <v>22</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="12">
-        <v>45852</v>
-      </c>
-      <c r="D14" s="12">
-        <v>45866</v>
-      </c>
-      <c r="E14" s="11">
-        <v>14</v>
+      <c r="D14" s="24">
+        <v>45845</v>
+      </c>
+      <c r="E14" s="23">
+        <v>7</v>
       </c>
       <c r="F14" s="15" t="s">
         <v>13</v>
@@ -847,20 +874,20 @@
       <c r="G14" s="7"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="20" t="s">
-        <v>23</v>
+      <c r="A15" s="18" t="s">
+        <v>29</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C15" s="12">
-        <v>45866</v>
+        <v>45845</v>
       </c>
       <c r="D15" s="12">
-        <v>45880</v>
+        <v>45852</v>
       </c>
       <c r="E15" s="11">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F15" s="15" t="s">
         <v>13</v>
@@ -868,13 +895,97 @@
       <c r="G15" s="7"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
+      <c r="A16" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="24">
+        <v>45852</v>
+      </c>
+      <c r="D16" s="24">
+        <v>45859</v>
+      </c>
+      <c r="E16" s="23">
+        <v>7</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="7"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A17" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="12">
+        <v>45859</v>
+      </c>
+      <c r="D17" s="12">
+        <v>45866</v>
+      </c>
+      <c r="E17" s="11">
+        <v>7</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="7"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A18" s="22" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="24">
+        <v>45866</v>
+      </c>
+      <c r="D18" s="24">
+        <v>45873</v>
+      </c>
+      <c r="E18" s="23">
+        <v>7</v>
+      </c>
+      <c r="F18" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="7"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A19" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="12">
+        <v>45873</v>
+      </c>
+      <c r="D19" s="12">
+        <v>45880</v>
+      </c>
+      <c r="E19" s="11">
+        <v>7</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="7"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A20" s="2"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>